<commit_message>
Hız karşılaştırma tablosu KTP sayfasına taşındı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Uk1bBjuLSuDCCE3kW34Mr
</commit_message>
<xml_diff>
--- a/KTP_18m_KITAS_Takograf_Kablo_Testi.xlsx
+++ b/KTP_18m_KITAS_Takograf_Kablo_Testi.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="KTP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hız Karşılaştırma" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="EMC Kaynakları" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sinyal Listesi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="EMC Kaynakları" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sinyal Listesi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0;-0.0;0.0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0;-0.0;0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +62,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <sz val="8"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -72,13 +72,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
+      <i val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="4">
@@ -125,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,30 +152,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -572,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -611,7 +599,7 @@
       <c r="B2" s="4" t="n"/>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>KTP-XXXX / Rev.02</t>
+          <t>KTP-XXXX / Rev.03</t>
         </is>
       </c>
       <c r="D2" s="6" t="n"/>
@@ -909,7 +897,7 @@
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>TÜM TESTLER EMC KAYNAKLARI AÇIKKEN YAPILACAKTIR. ('EMC Kaynakları' sayfası)</t>
+          <t>TÜM TESTLER EMC KAYNAKLARI AÇIKKEN YAPILACAKTIR. (Liste: 'EMC Kaynakları' sekmesi)</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
@@ -1061,7 +1049,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Hız değerleri 'Hız Karşılaştırma' sayfasına girilir, OK/NOK otomatik hesaplanır.</t>
+          <t>Hız değerleri bu sayfanın altındaki 'HIZ KARŞILAŞTIRMA TABLOSU'na girilir, OK/NOK otomatik hesaplanır.</t>
         </is>
       </c>
       <c r="D24" s="4" t="n"/>
@@ -1314,98 +1302,378 @@
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="n"/>
     </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>GENEL SONUÇ / NOTLAR:</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="5" t="inlineStr"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="6" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>Açıklama: Sarı hücreler test ekibi tarafından doldurulacaktır. Tolerans değerleri (±2 / ±3 km/h, cluster %10 + 4 km/h) öneridir; proje/regülasyon gereksinimleri ile teyit edilmelidir. TCO1 ID'si takograf DBC'sinden alınmıştır; EBS mesaj ID'leri J1939 standart değerleridir ve EBS DBC'si ile teyit edilmelidir.</t>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>HIZ KARŞILAŞTIRMA TABLOSU (Madde 2)</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Tolerans Takograf–EBS (± km/h):</t>
         </is>
       </c>
       <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
+      <c r="C40" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Cluster okuma payı (km/h):</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="4" t="n"/>
+      <c r="H40" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Hız (km/h)</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>Cluster (km/h)</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>Takograf TCO1 (km/h)</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>EBS (km/h)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>Fark Takograf–EBS (km/h)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="14" t="inlineStr">
+        <is>
+          <t>OK / NOK</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="16">
+        <f>IF(OR(C42="",D42=""),"",C42-D42)</f>
+        <v/>
+      </c>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="17">
+        <f>IF(OR(B42="",C42="",D42=""),"",IF(AND(ABS(C42-D42)&lt;=$C$40,B42&gt;=C42-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="16">
+        <f>IF(OR(C43="",D43=""),"",C43-D43)</f>
+        <v/>
+      </c>
+      <c r="G43" s="4" t="n"/>
+      <c r="H43" s="17">
+        <f>IF(OR(B43="",C43="",D43=""),"",IF(AND(ABS(C43-D43)&lt;=$C$40,B43&gt;=C43-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="16">
+        <f>IF(OR(C44="",D44=""),"",C44-D44)</f>
+        <v/>
+      </c>
+      <c r="G44" s="4" t="n"/>
+      <c r="H44" s="17">
+        <f>IF(OR(B44="",C44="",D44=""),"",IF(AND(ABS(C44-D44)&lt;=$C$40,B44&gt;=C44-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="16">
+        <f>IF(OR(C45="",D45=""),"",C45-D45)</f>
+        <v/>
+      </c>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="17">
+        <f>IF(OR(B45="",C45="",D45=""),"",IF(AND(ABS(C45-D45)&lt;=$C$40,B45&gt;=C45-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="15" t="n"/>
+      <c r="D46" s="15" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="16">
+        <f>IF(OR(C46="",D46=""),"",C46-D46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="17">
+        <f>IF(OR(B46="",C46="",D46=""),"",IF(AND(ABS(C46-D46)&lt;=$C$40,B46&gt;=C46-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="15" t="n"/>
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="16">
+        <f>IF(OR(C47="",D47=""),"",C47-D47)</f>
+        <v/>
+      </c>
+      <c r="G47" s="4" t="n"/>
+      <c r="H47" s="17">
+        <f>IF(OR(B47="",C47="",D47=""),"",IF(AND(ABS(C47-D47)&lt;=$C$40,B47&gt;=C47-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="16">
+        <f>IF(OR(C48="",D48=""),"",C48-D48)</f>
+        <v/>
+      </c>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="17">
+        <f>IF(OR(B48="",C48="",D48=""),"",IF(AND(ABS(C48-D48)&lt;=$C$40,B48&gt;=C48-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="15" t="n"/>
+      <c r="D49" s="15" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="16">
+        <f>IF(OR(C49="",D49=""),"",C49-D49)</f>
+        <v/>
+      </c>
+      <c r="G49" s="4" t="n"/>
+      <c r="H49" s="17">
+        <f>IF(OR(B49="",C49="",D49=""),"",IF(AND(ABS(C49-D49)&lt;=$C$40,B49&gt;=C49-$H$40),"OK","NOK"))</f>
+        <v/>
+      </c>
+      <c r="I49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
+        <is>
+          <t>OK şartı: |Takograf – EBS| ≤ tolerans VE Cluster ≥ Takograf – okuma payı. Sarı hücreler test ekibi tarafından doldurulur.</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>GENEL SONUÇ / NOTLAR:</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="n"/>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>Açıklama: Sarı hücreler test ekibi tarafından doldurulacaktır. Tolerans değerleri (±2 / ±3 km/h, cluster %10 + 4 km/h) öneridir; proje/regülasyon gereksinimleri ile teyit edilmelidir. TCO1 ID'si takograf DBC'sinden alınmıştır; EBS mesaj ID'leri J1939 standart değerleridir ve EBS DBC'si ile teyit edilmelidir.</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="4" t="n"/>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="59">
+  <mergeCells count="91">
     <mergeCell ref="C36:I36"/>
-    <mergeCell ref="C23:I23"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C32:I32"/>
     <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C38:I38"/>
-    <mergeCell ref="G8:H8"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="C19:I19"/>
-    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="D45:E45"/>
     <mergeCell ref="C28:I28"/>
-    <mergeCell ref="C13:I13"/>
-    <mergeCell ref="C18:I18"/>
-    <mergeCell ref="G7:H7"/>
     <mergeCell ref="C3:I3"/>
-    <mergeCell ref="C34:I34"/>
     <mergeCell ref="A17:I17"/>
-    <mergeCell ref="C24:I24"/>
-    <mergeCell ref="G6:H6"/>
     <mergeCell ref="C30:I30"/>
-    <mergeCell ref="C15:I15"/>
-    <mergeCell ref="C33:I33"/>
-    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="D48:E48"/>
     <mergeCell ref="C5:I5"/>
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="C14:I14"/>
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="C4:I4"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="C31:I31"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="C21:I21"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C23:I23"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="C18:I18"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="C20:I20"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="C29:I29"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="C32:I32"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="C24:I24"/>
+    <mergeCell ref="C33:I33"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C26:I26"/>
     <mergeCell ref="A26:A29"/>
     <mergeCell ref="C35:I35"/>
-    <mergeCell ref="C4:I4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C20:I20"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="C29:I29"/>
     <mergeCell ref="C10:I10"/>
     <mergeCell ref="C16:I16"/>
     <mergeCell ref="C25:I25"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A22:A25"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C31:I31"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C22:I22"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="A7:B8"/>
     <mergeCell ref="A11:B16"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C21:I21"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="C12:I12"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="F49:G49"/>
     <mergeCell ref="C2:I2"/>
-    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A40:B40"/>
     <mergeCell ref="C11:I11"/>
+    <mergeCell ref="C52:I52"/>
+    <mergeCell ref="A54:I54"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="C13:I13"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="C15:I15"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D44:E44"/>
     <mergeCell ref="C27:I27"/>
+    <mergeCell ref="F44:G44"/>
   </mergeCells>
+  <conditionalFormatting sqref="H42:I49">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"NOK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="C21 C25 C29 C33 C37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OK,NOK"</formula1>
@@ -1422,465 +1690,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="9" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>TCO1–EBS tolerans (± km/h)</t>
-        </is>
-      </c>
-      <c r="C1" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D1" s="16" t="inlineStr">
-        <is>
-          <t>← Parametreler öneridir (cluster sınırı ECE R39 mantığı: 0 ≤ Cluster–Gerçek hız ≤ %10 × hız + 4 km/h). Proje ile teyit edilecek.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>Cluster üst sınır oranı (× TCO1)</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Cluster üst sınır sabit (km/h)</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Cluster okuma toleransı (km/h)</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t>Hız Kademesi (km/h)</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>TCO1 Hızı ort. (km/h)</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>EBS Hızı ort. (km/h)</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
-        <is>
-          <t>Cluster Okunan (km/h)</t>
-        </is>
-      </c>
-      <c r="E6" s="18" t="inlineStr">
-        <is>
-          <t>GPS Hızı ops. (km/h)</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
-        <is>
-          <t>Fark TCO1–EBS (km/h)</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>Fark Cluster–TCO1 (km/h)</t>
-        </is>
-      </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>Cluster Üst Sınır (km/h)</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>Kesinti Sayısı</t>
-        </is>
-      </c>
-      <c r="J6" s="18" t="inlineStr">
-        <is>
-          <t>OK/NOK TCO1–EBS</t>
-        </is>
-      </c>
-      <c r="K6" s="18" t="inlineStr">
-        <is>
-          <t>OK/NOK Cluster</t>
-        </is>
-      </c>
-      <c r="L6" s="18" t="inlineStr">
-        <is>
-          <t>GENEL</t>
-        </is>
-      </c>
-      <c r="M6" s="18" t="inlineStr">
-        <is>
-          <t>Açıklama</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="21">
-        <f>IF(OR(B7="",C7=""),"",B7-C7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="21">
-        <f>IF(OR(B7="",D7=""),"",D7-B7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="21">
-        <f>IF(B7="","",B7+$C$2*B7+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="19">
-        <f>IF(F7="","",IF(AND(ABS(F7)&lt;=$C$1,OR(I7="",I7=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K7" s="19">
-        <f>IF(G7="","",IF(AND(G7&gt;=-$C$4,D7&lt;=H7),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L7" s="19">
-        <f>IF(OR(J7="",K7=""),"",IF(AND(J7="OK",K7="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M7" s="23" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="21">
-        <f>IF(OR(B8="",C8=""),"",B8-C8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="21">
-        <f>IF(OR(B8="",D8=""),"",D8-B8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="21">
-        <f>IF(B8="","",B8+$C$2*B8+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="19">
-        <f>IF(F8="","",IF(AND(ABS(F8)&lt;=$C$1,OR(I8="",I8=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K8" s="19">
-        <f>IF(G8="","",IF(AND(G8&gt;=-$C$4,D8&lt;=H8),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L8" s="19">
-        <f>IF(OR(J8="",K8=""),"",IF(AND(J8="OK",K8="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M8" s="23" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="21">
-        <f>IF(OR(B9="",C9=""),"",B9-C9)</f>
-        <v/>
-      </c>
-      <c r="G9" s="21">
-        <f>IF(OR(B9="",D9=""),"",D9-B9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="21">
-        <f>IF(B9="","",B9+$C$2*B9+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I9" s="22" t="n"/>
-      <c r="J9" s="19">
-        <f>IF(F9="","",IF(AND(ABS(F9)&lt;=$C$1,OR(I9="",I9=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K9" s="19">
-        <f>IF(G9="","",IF(AND(G9&gt;=-$C$4,D9&lt;=H9),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L9" s="19">
-        <f>IF(OR(J9="",K9=""),"",IF(AND(J9="OK",K9="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M9" s="23" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-      <c r="F10" s="21">
-        <f>IF(OR(B10="",C10=""),"",B10-C10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="21">
-        <f>IF(OR(B10="",D10=""),"",D10-B10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="21">
-        <f>IF(B10="","",B10+$C$2*B10+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I10" s="22" t="n"/>
-      <c r="J10" s="19">
-        <f>IF(F10="","",IF(AND(ABS(F10)&lt;=$C$1,OR(I10="",I10=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K10" s="19">
-        <f>IF(G10="","",IF(AND(G10&gt;=-$C$4,D10&lt;=H10),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L10" s="19">
-        <f>IF(OR(J10="",K10=""),"",IF(AND(J10="OK",K10="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M10" s="23" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="n">
-        <v>50</v>
-      </c>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="21">
-        <f>IF(OR(B11="",C11=""),"",B11-C11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="21">
-        <f>IF(OR(B11="",D11=""),"",D11-B11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="21">
-        <f>IF(B11="","",B11+$C$2*B11+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I11" s="22" t="n"/>
-      <c r="J11" s="19">
-        <f>IF(F11="","",IF(AND(ABS(F11)&lt;=$C$1,OR(I11="",I11=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K11" s="19">
-        <f>IF(G11="","",IF(AND(G11&gt;=-$C$4,D11&lt;=H11),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L11" s="19">
-        <f>IF(OR(J11="",K11=""),"",IF(AND(J11="OK",K11="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M11" s="23" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="n">
-        <v>60</v>
-      </c>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="21">
-        <f>IF(OR(B12="",C12=""),"",B12-C12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="21">
-        <f>IF(OR(B12="",D12=""),"",D12-B12)</f>
-        <v/>
-      </c>
-      <c r="H12" s="21">
-        <f>IF(B12="","",B12+$C$2*B12+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I12" s="22" t="n"/>
-      <c r="J12" s="19">
-        <f>IF(F12="","",IF(AND(ABS(F12)&lt;=$C$1,OR(I12="",I12=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K12" s="19">
-        <f>IF(G12="","",IF(AND(G12&gt;=-$C$4,D12&lt;=H12),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L12" s="19">
-        <f>IF(OR(J12="",K12=""),"",IF(AND(J12="OK",K12="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M12" s="23" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="n">
-        <v>70</v>
-      </c>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="21">
-        <f>IF(OR(B13="",C13=""),"",B13-C13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="21">
-        <f>IF(OR(B13="",D13=""),"",D13-B13)</f>
-        <v/>
-      </c>
-      <c r="H13" s="21">
-        <f>IF(B13="","",B13+$C$2*B13+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I13" s="22" t="n"/>
-      <c r="J13" s="19">
-        <f>IF(F13="","",IF(AND(ABS(F13)&lt;=$C$1,OR(I13="",I13=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K13" s="19">
-        <f>IF(G13="","",IF(AND(G13&gt;=-$C$4,D13&lt;=H13),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L13" s="19">
-        <f>IF(OR(J13="",K13=""),"",IF(AND(J13="OK",K13="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M13" s="23" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="n">
-        <v>80</v>
-      </c>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-      <c r="F14" s="21">
-        <f>IF(OR(B14="",C14=""),"",B14-C14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="21">
-        <f>IF(OR(B14="",D14=""),"",D14-B14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="21">
-        <f>IF(B14="","",B14+$C$2*B14+$C$3)</f>
-        <v/>
-      </c>
-      <c r="I14" s="22" t="n"/>
-      <c r="J14" s="19">
-        <f>IF(F14="","",IF(AND(ABS(F14)&lt;=$C$1,OR(I14="",I14=0)),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="K14" s="19">
-        <f>IF(G14="","",IF(AND(G14&gt;=-$C$4,D14&lt;=H14),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="L14" s="19">
-        <f>IF(OR(J14="",K14=""),"",IF(AND(J14="OK",K14="OK"),"OK","NOK"))</f>
-        <v/>
-      </c>
-      <c r="M14" s="23" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Örnek: 50 km/h kademesi → TCO1 50,4 / EBS 49,8 / Cluster 53 → TCO1–EBS 0,6 (OK); Cluster–TCO1 2,6, üst sınır 59,4 (OK) → GENEL OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>Mavi/sarı hücreler ölçümden girilir; farklar ve OK/NOK formülle hesaplanır. Kesinti Sayısı: TCO1 &gt; 150 ms boşluk veya hızın anlık 0'a / geçersiz değere düşmesi.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="J7:J14">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"NOK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K14">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
-      <formula>"NOK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L14">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="0">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
-      <formula>"NOK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1892,27 +1701,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>EMC Kaynağı / Tüketici</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>Test Sırasında AÇIK (☐/☑)</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>Açma-Kapama Geçişinde Hız Sinyali Etkilendi mi? (E/H)</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Not</t>
         </is>
@@ -2217,7 +2026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2237,42 +2046,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Kaynak ECU</t>
         </is>
       </c>
-      <c r="B1" s="24" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Mesaj</t>
         </is>
       </c>
-      <c r="C1" s="24" t="inlineStr">
+      <c r="C1" s="19" t="inlineStr">
         <is>
           <t>CAN ID (29-bit)</t>
         </is>
       </c>
-      <c r="D1" s="24" t="inlineStr">
+      <c r="D1" s="19" t="inlineStr">
         <is>
           <t>Sinyal</t>
         </is>
       </c>
-      <c r="E1" s="24" t="inlineStr">
+      <c r="E1" s="19" t="inlineStr">
         <is>
           <t>Byte / Bit (Intel)</t>
         </is>
       </c>
-      <c r="F1" s="24" t="inlineStr">
+      <c r="F1" s="19" t="inlineStr">
         <is>
           <t>Ölçek / Birim</t>
         </is>
       </c>
-      <c r="G1" s="24" t="inlineStr">
+      <c r="G1" s="19" t="inlineStr">
         <is>
           <t>Periyot</t>
         </is>
       </c>
-      <c r="H1" s="24" t="inlineStr">
+      <c r="H1" s="19" t="inlineStr">
         <is>
           <t>Kontrol Amacı</t>
         </is>
@@ -2294,7 +2103,7 @@
           <t>0x0CFE6CEE</t>
         </is>
       </c>
-      <c r="D2" s="25" t="inlineStr">
+      <c r="D2" s="20" t="inlineStr">
         <is>
           <t>TachographVehicleSpeed</t>
         </is>
@@ -2657,7 +2466,7 @@
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>* EBS mesaj ID'leri SAE J1939 standart değerleridir (SA 0x0B = fren sistemi); araç EBS DBC dosyası ile teyit edilmelidir. TCO1/VDHR ID'leri takograf DBC'sinden alınmıştır (DBC ID – 0x80000000).</t>
         </is>

</xml_diff>

<commit_message>
KTP: Sonuç satırları test ekibi için boş bırakıldı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Uk1bBjuLSuDCCE3kW34Mr
</commit_message>
<xml_diff>
--- a/KTP_18m_KITAS_Takograf_Kablo_Testi.xlsx
+++ b/KTP_18m_KITAS_Takograf_Kablo_Testi.xlsx
@@ -544,7 +544,7 @@
       <c r="B2" s="4" t="n"/>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>KTP-XXXX / Rev.04</t>
+          <t>KTP-XXXX / Rev.05</t>
         </is>
       </c>
       <c r="D2" s="6" t="n"/>
@@ -916,17 +916,13 @@
           <t>SONUÇ</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Takograf, EBS ve cluster hız değerleri 0 km/h görülür.</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="n"/>
@@ -992,17 +988,13 @@
           <t>SONUÇ</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Her hızda cluster, takograf ve EBS hız değerleri kaydedilir.</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-      <c r="I24" s="4" t="n"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="n"/>
@@ -1068,17 +1060,13 @@
           <t>SONUÇ</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Takograf ve EBS hız grafikleri üst üste çakışır, kesinti görülmez.</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="n"/>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="n"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="n"/>
@@ -1144,17 +1132,13 @@
           <t>SONUÇ</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Hız sinyali kesintisiz devam eder.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="n"/>
-      <c r="F32" s="4" t="n"/>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="n"/>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="6" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="n"/>
@@ -1220,17 +1204,13 @@
           <t>SONUÇ</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Hata kaydı oluşmaz.</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="n"/>

</xml_diff>